<commit_message>
feat: standardize location to 20 accident places, retain original workGroup, map workMethod to 9x9, and update all records
</commit_message>
<xml_diff>
--- a/samples/부적합사항대장_샘플.xlsx
+++ b/samples/부적합사항대장_샘플.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="973" uniqueCount="711">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="975" uniqueCount="713">
   <si>
     <t>No</t>
   </si>
@@ -685,7 +685,7 @@
     <t>안전장치의 기능 제거</t>
   </si>
   <si>
-    <t>토공사/기초공사</t>
+    <t>토공사</t>
   </si>
   <si>
     <t>띠장(수평재)</t>
@@ -718,6 +718,9 @@
     <t>보호구 미착용·잘못 사용</t>
   </si>
   <si>
+    <t>기초공사</t>
+  </si>
+  <si>
     <t>장선</t>
   </si>
   <si>
@@ -748,42 +751,39 @@
     <t>기계·기구의 잘못 사용</t>
   </si>
   <si>
+    <t>가새</t>
+  </si>
+  <si>
+    <t>안전보건규칙 제68조</t>
+  </si>
+  <si>
+    <t>작업시설 미설치</t>
+  </si>
+  <si>
+    <t>계획: 시공계획서 안전대책 미수립/미승인</t>
+  </si>
+  <si>
+    <t>토목/인프라</t>
+  </si>
+  <si>
+    <t>준공 및 부대토목 단계</t>
+  </si>
+  <si>
+    <t>설비·장치</t>
+  </si>
+  <si>
+    <t>미끄러짐/접질림</t>
+  </si>
+  <si>
+    <t>작업환경의 결함 (조명·환기·소음 등)</t>
+  </si>
+  <si>
+    <t>운전 중인 기계장치 점검·손질</t>
+  </si>
+  <si>
     <t>철골공사</t>
   </si>
   <si>
-    <t>가새</t>
-  </si>
-  <si>
-    <t>안전보건규칙 제68조</t>
-  </si>
-  <si>
-    <t>작업시설 미설치</t>
-  </si>
-  <si>
-    <t>계획: 시공계획서 안전대책 미수립/미승인</t>
-  </si>
-  <si>
-    <t>토목/인프라</t>
-  </si>
-  <si>
-    <t>준공 및 부대토목 단계</t>
-  </si>
-  <si>
-    <t>설비·장치</t>
-  </si>
-  <si>
-    <t>미끄러짐/접질림</t>
-  </si>
-  <si>
-    <t>작업환경의 결함 (조명·환기·소음 등)</t>
-  </si>
-  <si>
-    <t>운전 중인 기계장치 점검·손질</t>
-  </si>
-  <si>
-    <t>조적/미장/방수공사</t>
-  </si>
-  <si>
     <t>벽이음</t>
   </si>
   <si>
@@ -811,7 +811,7 @@
     <t>불안전한 속도 조작</t>
   </si>
   <si>
-    <t>마감/수장공사</t>
+    <t>양중공사</t>
   </si>
   <si>
     <t>안전보건규칙 제63조</t>
@@ -832,7 +832,7 @@
     <t>위험물 취급 부주의</t>
   </si>
   <si>
-    <t>기계설비공사</t>
+    <t>마감공사</t>
   </si>
   <si>
     <t>안전난간</t>
@@ -853,7 +853,7 @@
     <t>불안전한 상태 방치</t>
   </si>
   <si>
-    <t>전기/통신공사</t>
+    <t>설비·전기공사</t>
   </si>
   <si>
     <t>발끝막이판</t>
@@ -877,7 +877,7 @@
     <t>불안전한 자세·동작</t>
   </si>
   <si>
-    <t>해체/철거공사</t>
+    <t>해체공사</t>
   </si>
   <si>
     <t>클램프·연결철물</t>
@@ -901,6 +901,9 @@
     <t>감독 및 연락·신호 불충분</t>
   </si>
   <si>
+    <t>토목·조경·포장</t>
+  </si>
+  <si>
     <t>받침철물</t>
   </si>
   <si>
@@ -911,6 +914,9 @@
   </si>
   <si>
     <t>질식/중독 등</t>
+  </si>
+  <si>
+    <t>공통</t>
   </si>
   <si>
     <t>주틀</t>
@@ -3875,7 +3881,7 @@
       <formula1>분류기준!$D$2:$D$51</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="공종" prompt="목록에서 선택하거나 직접 입력하세요" sqref="H3:H19">
-      <formula1>분류기준!$H$2:$H$40</formula1>
+      <formula1>분류기준!$H$2:$H$42</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="작업방법" prompt="목록에서 선택하거나 직접 입력하세요" sqref="I3:I19">
       <formula1>분류기준!$I$2:$I$40</formula1>
@@ -4479,7 +4485,7 @@
     <col min="5" max="5" width="36" customWidth="1"/>
     <col min="6" max="6" width="35.2" customWidth="1"/>
     <col min="7" max="7" width="25.6" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="8" max="8" width="12.8" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
     <col min="10" max="10" width="20.8" customWidth="1"/>
     <col min="11" max="11" width="36" customWidth="1"/>
@@ -4656,19 +4662,19 @@
         <v>232</v>
       </c>
       <c r="H4" s="23" t="s">
-        <v>70</v>
+        <v>233</v>
       </c>
       <c r="I4" s="23" t="s">
         <v>71</v>
       </c>
       <c r="J4" s="23" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="K4" s="23" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="L4" s="23" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="M4" s="23" t="s">
         <v>78</v>
@@ -4677,30 +4683,30 @@
         <v>58</v>
       </c>
       <c r="P4" s="23" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B5" s="23" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F5" s="23" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="G5" s="23" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="H5" s="23" t="s">
-        <v>243</v>
+        <v>70</v>
       </c>
       <c r="I5" s="23" t="s">
         <v>124</v>
@@ -4900,11 +4906,14 @@
       <c r="G11" s="23" t="s">
         <v>293</v>
       </c>
+      <c r="H11" s="23" t="s">
+        <v>294</v>
+      </c>
       <c r="J11" s="23" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="K11" s="23" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L11" s="23" t="s">
         <v>77</v>
@@ -4915,259 +4924,262 @@
     </row>
     <row r="12" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D12" s="23" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="G12" s="23" t="s">
         <v>193</v>
       </c>
+      <c r="H12" s="23" t="s">
+        <v>299</v>
+      </c>
       <c r="J12" s="23" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="K12" s="23" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="L12" s="23" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="M12" s="23" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
     </row>
     <row r="13" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D13" s="23" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="J13" s="23" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="K13" s="23" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="L13" s="23" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="M13" s="23" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="14" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D14" s="23" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="J14" s="23" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="K14" s="23" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="L14" s="23" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="M14" s="23" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="15" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D15" s="23" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="J15" s="23" t="s">
         <v>183</v>
       </c>
       <c r="K15" s="23" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="L15" s="23" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="M15" s="23" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="16" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D16" s="23" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="J16" s="23" t="s">
         <v>184</v>
       </c>
       <c r="K16" s="23" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="L16" s="23" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="M16" s="23" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="17" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D17" s="23" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="E17" s="23" t="s">
         <v>193</v>
       </c>
       <c r="J17" s="23" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="K17" s="23" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="L17" s="23" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="M17" s="23" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="18" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D18" s="23" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="J18" s="23" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="K18" s="23" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L18" s="23" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="M18" s="23" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="19" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D19" s="23" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="J19" s="23" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="K19" s="23" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="L19" s="23" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="M19" s="23" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="20" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D20" s="23" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="J20" s="23" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="K20" s="23" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="L20" s="23" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="M20" s="23" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="21" spans="4:12" x14ac:dyDescent="0.25">
       <c r="D21" s="23" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="J21" s="23" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="K21" s="23" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="L21" s="23" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
     <row r="22" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J22" s="23" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="K22" s="23" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="L22" s="23" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
     </row>
     <row r="23" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J23" s="23" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="K23" s="23" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="L23" s="23" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="24" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J24" s="23" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="K24" s="23" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="L24" s="23" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="25" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J25" s="23" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="K25" s="23" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="L25" s="23" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="26" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J26" s="23" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="K26" s="23" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="L26" s="23" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="27" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J27" s="23" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="K27" s="23" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="L27" s="23" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
     </row>
     <row r="28" spans="10:12" x14ac:dyDescent="0.25">
@@ -5175,98 +5187,98 @@
         <v>136</v>
       </c>
       <c r="K28" s="23" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="L28" s="23" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
     </row>
     <row r="29" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J29" s="23" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="K29" s="23" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="L29" s="23" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
     </row>
     <row r="30" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J30" s="23" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="K30" s="23" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="L30" s="23" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
     </row>
     <row r="31" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J31" s="23" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="K31" s="23" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="L31" s="23" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
     </row>
     <row r="32" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J32" s="23" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="K32" s="23" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="L32" s="23" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
     </row>
     <row r="33" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J33" s="23" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="K33" s="23" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="L33" s="23" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="34" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J34" s="23" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="K34" s="23" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="L34" s="23" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
     </row>
     <row r="35" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J35" s="23" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="K35" s="23" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="L35" s="23" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="36" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J36" s="23" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="K36" s="23" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="L36" s="23" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
     </row>
     <row r="37" spans="10:12" x14ac:dyDescent="0.25">
@@ -5274,51 +5286,51 @@
         <v>144</v>
       </c>
       <c r="K37" s="23" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="L37" s="23" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
     </row>
     <row r="38" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J38" s="23" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="K38" s="23" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="L38" s="23" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
     </row>
     <row r="39" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J39" s="23" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="K39" s="23" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="L39" s="23" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="40" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J40" s="23" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="K40" s="23" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="L40" s="23" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
     </row>
     <row r="41" spans="10:11" x14ac:dyDescent="0.25">
       <c r="J41" s="23" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="K41" s="23" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
     </row>
     <row r="42" spans="10:11" x14ac:dyDescent="0.25">
@@ -5326,370 +5338,370 @@
         <v>187</v>
       </c>
       <c r="K42" s="23" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
     </row>
     <row r="43" spans="10:11" x14ac:dyDescent="0.25">
       <c r="J43" s="23" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="K43" s="23" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
     </row>
     <row r="44" spans="10:11" x14ac:dyDescent="0.25">
       <c r="J44" s="23" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="K44" s="23" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="45" spans="10:11" x14ac:dyDescent="0.25">
       <c r="J45" s="23" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="K45" s="23" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
     </row>
     <row r="46" spans="10:11" x14ac:dyDescent="0.25">
       <c r="J46" s="23" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="K46" s="23" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="47" spans="10:11" x14ac:dyDescent="0.25">
       <c r="J47" s="23" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="K47" s="23" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
     </row>
     <row r="48" spans="10:11" x14ac:dyDescent="0.25">
       <c r="J48" s="23" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="K48" s="23" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="49" spans="10:11" x14ac:dyDescent="0.25">
       <c r="J49" s="23" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="K49" s="23" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
     </row>
     <row r="50" spans="10:11" x14ac:dyDescent="0.25">
       <c r="J50" s="23" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="K50" s="23" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
     </row>
     <row r="51" spans="10:11" x14ac:dyDescent="0.25">
       <c r="J51" s="23" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="K51" s="23" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
     </row>
     <row r="52" spans="10:11" x14ac:dyDescent="0.25">
       <c r="J52" s="23" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="K52" s="23" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
     </row>
     <row r="53" spans="10:11" x14ac:dyDescent="0.25">
       <c r="J53" s="23" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="K53" s="23" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="54" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J54" s="23" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
     </row>
     <row r="55" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J55" s="23" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
     </row>
     <row r="56" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J56" s="23" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
     </row>
     <row r="57" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J57" s="23" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
     </row>
     <row r="58" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J58" s="23" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
     <row r="59" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J59" s="23" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
     </row>
     <row r="60" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J60" s="23" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
     <row r="61" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J61" s="23" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
     </row>
     <row r="62" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J62" s="23" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="63" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J63" s="23" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
     </row>
     <row r="64" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J64" s="23" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="65" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J65" s="23" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
     </row>
     <row r="66" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J66" s="23" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
     </row>
     <row r="67" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J67" s="23" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="68" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J68" s="23" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
     </row>
     <row r="69" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J69" s="23" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
     </row>
     <row r="70" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J70" s="23" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
     </row>
     <row r="71" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J71" s="23" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
     </row>
     <row r="72" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J72" s="23" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
     </row>
     <row r="73" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J73" s="23" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
     </row>
     <row r="74" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J74" s="23" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
     </row>
     <row r="75" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J75" s="23" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
     </row>
     <row r="76" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J76" s="23" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
     </row>
     <row r="77" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J77" s="23" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
     </row>
     <row r="78" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J78" s="23" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
     </row>
     <row r="79" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J79" s="23" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
     </row>
     <row r="80" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J80" s="23" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
     </row>
     <row r="81" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J81" s="23" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
     </row>
     <row r="82" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J82" s="23" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
     </row>
     <row r="83" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J83" s="23" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
     </row>
     <row r="84" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J84" s="23" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
     </row>
     <row r="85" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J85" s="23" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
     </row>
     <row r="86" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J86" s="23" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
     </row>
     <row r="87" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J87" s="23" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
     </row>
     <row r="88" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J88" s="23" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
     </row>
     <row r="89" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J89" s="23" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
     </row>
     <row r="90" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J90" s="23" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
     </row>
     <row r="91" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J91" s="23" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
     </row>
     <row r="92" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J92" s="23" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
     </row>
     <row r="93" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J93" s="23" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
     </row>
     <row r="94" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J94" s="23" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
     </row>
     <row r="95" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J95" s="23" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
     </row>
     <row r="96" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J96" s="23" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
     </row>
     <row r="97" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J97" s="23" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="98" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J98" s="23" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
     </row>
     <row r="99" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J99" s="23" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
     </row>
     <row r="100" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J100" s="23" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
     </row>
     <row r="101" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J101" s="23" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
     </row>
     <row r="102" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J102" s="23" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
     </row>
     <row r="103" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J103" s="23" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
     </row>
     <row r="104" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J104" s="23" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
     </row>
     <row r="105" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J105" s="23" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
     </row>
     <row r="106" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J106" s="23" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="107" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J107" s="23" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="108" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J108" s="23" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
     </row>
     <row r="109" spans="10:10" x14ac:dyDescent="0.25">
@@ -5699,12 +5711,12 @@
     </row>
     <row r="110" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J110" s="23" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
     </row>
     <row r="111" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J111" s="23" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
     <row r="112" spans="10:10" x14ac:dyDescent="0.25">
@@ -5714,32 +5726,32 @@
     </row>
     <row r="113" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J113" s="23" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
     </row>
     <row r="114" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J114" s="23" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
     </row>
     <row r="115" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J115" s="23" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
     </row>
     <row r="116" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J116" s="23" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="117" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J117" s="23" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
     </row>
     <row r="118" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J118" s="23" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
     </row>
     <row r="119" spans="10:10" x14ac:dyDescent="0.25">
@@ -5749,62 +5761,62 @@
     </row>
     <row r="120" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J120" s="23" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="121" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J121" s="23" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
     <row r="122" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J122" s="23" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
     </row>
     <row r="123" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J123" s="23" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row r="124" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J124" s="23" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
     </row>
     <row r="125" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J125" s="23" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="126" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J126" s="23" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="127" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J127" s="23" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="128" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J128" s="23" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="129" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J129" s="23" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="130" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J130" s="23" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
     </row>
     <row r="131" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J131" s="23" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
     </row>
     <row r="132" spans="10:10" x14ac:dyDescent="0.25">
@@ -5814,17 +5826,17 @@
     </row>
     <row r="133" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J133" s="23" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
     </row>
     <row r="134" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J134" s="23" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="135" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J135" s="23" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="136" spans="10:10" x14ac:dyDescent="0.25">
@@ -5834,22 +5846,22 @@
     </row>
     <row r="137" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J137" s="23" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
     <row r="138" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J138" s="23" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="139" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J139" s="23" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
     </row>
     <row r="140" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J140" s="23" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="141" spans="10:10" x14ac:dyDescent="0.25">
@@ -5859,137 +5871,137 @@
     </row>
     <row r="142" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J142" s="23" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="143" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J143" s="23" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
     </row>
     <row r="144" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J144" s="23" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
     </row>
     <row r="145" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J145" s="23" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
     <row r="146" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J146" s="23" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
     </row>
     <row r="147" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J147" s="23" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
     </row>
     <row r="148" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J148" s="23" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
     </row>
     <row r="149" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J149" s="23" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
     </row>
     <row r="150" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J150" s="23" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
     </row>
     <row r="151" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J151" s="23" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
     </row>
     <row r="152" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J152" s="23" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
     </row>
     <row r="153" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J153" s="23" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
     </row>
     <row r="154" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J154" s="23" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
     </row>
     <row r="155" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J155" s="23" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
     </row>
     <row r="156" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J156" s="23" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
     </row>
     <row r="157" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J157" s="23" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
     </row>
     <row r="158" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J158" s="23" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
     </row>
     <row r="159" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J159" s="23" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
     </row>
     <row r="160" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J160" s="23" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
     </row>
     <row r="161" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J161" s="23" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
     </row>
     <row r="162" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J162" s="23" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
     </row>
     <row r="163" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J163" s="23" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
     </row>
     <row r="164" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J164" s="23" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
     </row>
     <row r="165" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J165" s="23" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
     </row>
     <row r="166" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J166" s="23" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
     </row>
     <row r="167" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J167" s="23" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
     </row>
     <row r="168" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J168" s="23" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
     </row>
   </sheetData>
@@ -6012,22 +6024,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="24" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="B1" s="24" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="C1" s="24" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="D1" s="24" t="s">
         <v>206</v>
       </c>
       <c r="E1" s="24" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="F1" s="24" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -6038,16 +6050,16 @@
         <v>182</v>
       </c>
       <c r="C2" s="25" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D2" s="25" t="s">
         <v>215</v>
       </c>
       <c r="E2" s="25" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="F2" s="25" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -6055,19 +6067,19 @@
         <v>88</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C3" s="25" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D3" s="25" t="s">
         <v>224</v>
       </c>
       <c r="E3" s="25" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="F3" s="25" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -6078,16 +6090,16 @@
         <v>50</v>
       </c>
       <c r="C4" s="25" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D4" s="25" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E4" s="25" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="F4" s="25" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -6095,19 +6107,19 @@
         <v>88</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="C5" s="25" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D5" s="25" t="s">
         <v>245</v>
       </c>
       <c r="E5" s="25" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="F5" s="25" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -6118,16 +6130,16 @@
         <v>109</v>
       </c>
       <c r="C6" s="25" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D6" s="25" t="s">
         <v>256</v>
       </c>
       <c r="E6" s="25" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="F6" s="25" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -6138,16 +6150,16 @@
         <v>117</v>
       </c>
       <c r="C7" s="25" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D7" s="25" t="s">
         <v>265</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="F7" s="25" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -6158,16 +6170,16 @@
         <v>91</v>
       </c>
       <c r="C8" s="25" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D8" s="25" t="s">
         <v>273</v>
       </c>
       <c r="E8" s="25" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="F8" s="25" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -6178,16 +6190,16 @@
         <v>272</v>
       </c>
       <c r="C9" s="25" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D9" s="25" t="s">
         <v>280</v>
       </c>
       <c r="E9" s="25" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="F9" s="25" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -6198,16 +6210,16 @@
         <v>130</v>
       </c>
       <c r="C10" s="25" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D10" s="25" t="s">
         <v>288</v>
       </c>
       <c r="E10" s="25" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="F10" s="25" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -6215,19 +6227,19 @@
         <v>88</v>
       </c>
       <c r="B11" s="25" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C11" s="25" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D11" s="25" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E11" s="25" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="F11" s="25" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -6235,19 +6247,19 @@
         <v>88</v>
       </c>
       <c r="B12" s="25" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="C12" s="25" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="D12" s="25" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="E12" s="25" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="F12" s="25" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -6258,16 +6270,16 @@
         <v>190</v>
       </c>
       <c r="C13" s="25" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D13" s="25" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E13" s="25" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="F13" s="25" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -6275,19 +6287,19 @@
         <v>88</v>
       </c>
       <c r="B14" s="25" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="C14" s="25" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="D14" s="25" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="E14" s="25" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="F14" s="25" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -6295,19 +6307,19 @@
         <v>88</v>
       </c>
       <c r="B15" s="25" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D15" s="25" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E15" s="25" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="F15" s="25" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -6315,384 +6327,384 @@
         <v>88</v>
       </c>
       <c r="B16" s="25" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="D16" s="25" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="E16" s="25" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="F16" s="25" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="25" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="B17" s="25" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D17" s="25" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="E17" s="25" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="F17" s="25" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="25" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="B18" s="25" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D18" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E18" s="25" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="F18" s="25" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="B19" s="25" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D19" s="25" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="E19" s="25" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="F19" s="25" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="25" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="B20" s="25" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="D20" s="25" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="E20" s="25" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="F20" s="25" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="25" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="B21" s="25" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="D21" s="25" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="E21" s="25" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="F21" s="25" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="25" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="B22" s="25" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="E22" s="25" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="F22" s="25" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="25" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="B23" s="25" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="C23" s="25" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="E23" s="25" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="F23" s="25" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="25" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="B24" s="25" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="C24" s="25" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="D24" s="25" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="E24" s="25" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="F24" s="25" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="25" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="B25" s="25" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="C25" s="25" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="D25" s="25" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="E25" s="25" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="F25" s="25" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="25" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="B26" s="25" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="C26" s="25" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="D26" s="25" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="E26" s="25" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="F26" s="25" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="25" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="B27" s="25" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="C27" s="25" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D27" s="25" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="E27" s="25" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="F27" s="25" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="25" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="B28" s="25" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="C28" s="25" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="D28" s="25" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="E28" s="25" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="F28" s="25" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="25" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="B29" s="25" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="C29" s="25" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="D29" s="25" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="E29" s="25" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="F29" s="25" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="25" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="B30" s="25" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="C30" s="25" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="D30" s="25" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="E30" s="25" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="F30" s="25" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="25" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="B31" s="25" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="C31" s="25" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="D31" s="25" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="E31" s="25" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="F31" s="25" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="25" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="B32" s="25" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="C32" s="25" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="D32" s="25" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E32" s="25" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="F32" s="25" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="25" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="B33" s="25" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="C33" s="25" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="D33" s="25" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="E33" s="25" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="F33" s="25" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="25" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="B34" s="25" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="C34" s="25" t="s">
         <v>284</v>
       </c>
       <c r="D34" s="25" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="E34" s="25" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="F34" s="25" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="25" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="B35" s="25" t="s">
         <v>172</v>
@@ -6701,213 +6713,213 @@
         <v>284</v>
       </c>
       <c r="D35" s="25" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="E35" s="25" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="F35" s="25" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="25" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="B36" s="25" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="C36" s="25" t="s">
         <v>284</v>
       </c>
       <c r="D36" s="25" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="E36" s="25" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="F36" s="25" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="25" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="B37" s="25" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="C37" s="25" t="s">
         <v>284</v>
       </c>
       <c r="D37" s="25" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E37" s="25" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="F37" s="25" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="25" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="B38" s="25" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="C38" s="25" t="s">
         <v>284</v>
       </c>
       <c r="D38" s="25" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="E38" s="25" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
       <c r="F38" s="25" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="25" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="B39" s="25" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="C39" s="25" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="D39" s="25" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="E39" s="25" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="F39" s="25" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="25" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="B40" s="25" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
       <c r="C40" s="25" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
       <c r="D40" s="25" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="E40" s="25" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="F40" s="25" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="25" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="B41" s="25" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="C41" s="25" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="D41" s="25" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="E41" s="25" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="F41" s="25" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="25" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="B42" s="25" t="s">
         <v>101</v>
       </c>
       <c r="C42" s="25" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="D42" s="25" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="E42" s="25" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="F42" s="25" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="25" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="B43" s="25" t="s">
         <v>136</v>
       </c>
       <c r="C43" s="25" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D43" s="25" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="E43" s="25" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="F43" s="25" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="25" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="B44" s="25" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="C44" s="25" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="D44" s="25" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="E44" s="25" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="F44" s="25" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="25" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="B45" s="25" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="C45" s="25" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="D45" s="25" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="E45" s="25" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="F45" s="25" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -6915,199 +6927,199 @@
         <v>149</v>
       </c>
       <c r="B46" s="25" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="C46" s="25" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D46" s="25" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="E46" s="25" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="F46" s="25" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="25" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="B47" s="25" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="C47" s="25" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="D47" s="25" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="E47" s="25" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="F47" s="25" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="25" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="B48" s="25" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="C48" s="25" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="D48" s="25" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="E48" s="25" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="F48" s="25" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="25" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="B49" s="25" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="C49" s="25" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="D49" s="25" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="E49" s="25" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="F49" s="25" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="25" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="B50" s="25" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="C50" s="25" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="D50" s="25" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="E50" s="25" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="F50" s="25" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="25" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="B51" s="25" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="C51" s="25" t="s">
         <v>193</v>
       </c>
       <c r="D51" s="25" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="E51" s="25" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="F51" s="25" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="25" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="B52" s="25" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="C52" s="25" t="s">
         <v>193</v>
       </c>
       <c r="D52" s="25" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="E52" s="25" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="F52" s="25" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="25" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="B53" s="25" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="C53" s="25" t="s">
         <v>193</v>
       </c>
       <c r="D53" s="25" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="E53" s="25" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="F53" s="25" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="25" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="B54" s="25" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="C54" s="25" t="s">
         <v>193</v>
       </c>
       <c r="D54" s="25" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="E54" s="25" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="F54" s="25" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="25" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="B55" s="25" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="C55" s="25" t="s">
         <v>193</v>
       </c>
       <c r="D55" s="25" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E55" s="25" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="F55" s="25" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
     </row>
   </sheetData>

</xml_diff>